<commit_message>
Excel readers: numbers stored as text, square blocks of series
Numbers stored as text are read as numbers, and a square block of series
takes its direction from the x range (x in a row gives one series per row),
as Python PySD. Fixes #11.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/data/sample.xlsx
+++ b/test/data/sample.xlsx
@@ -17,6 +17,9 @@
     <definedName name="xs">Data!$H$2:$H$6</definedName>
     <definedName name="ys">Data!$I$2:$I$6</definedName>
     <definedName name="ys2">Data!$I$2:$J$6</definedName>
+    <definedName name="xs_row">Data!$B$13:$C$13</definedName>
+    <definedName name="ys_square">Data!$B$14:$C$15</definedName>
+    <definedName name="text_param">Data!$E$2</definedName>
     <definedName name="local_param" localSheetId="0">Data!$C$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -422,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:J11"/>
+  <dimension ref="B2:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -432,6 +435,11 @@
       <c r="C2" t="n">
         <v>7</v>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
       <c r="F2" t="n">
         <v>10</v>
       </c>
@@ -556,6 +564,30 @@
       </c>
       <c r="F11" t="n">
         <v>40</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="n">
+        <v>10</v>
+      </c>
+      <c r="C15" t="n">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>